<commit_message>
v15.0.0: new toolkit packages, Austin setup samples, live previews
Hosts ctc-chapter-setup 1.6.0 (now a plugin, eight questions in one
message), ctc-newsletter 2.5.1 and ctc-partner-map 2.2.0. Install uploads
all three as plugins. Copy follows the new skills: assembly needs both
files, picks two to four opportunities, harvest companion file, last
month's opportunities file, LinkedIn asked every run, partner map once.
Austin settings and plan replace the Denver samples; registry sample from
2.5.1; partner map rebuilt with 2.2.0.

Previews open the file itself: Excel-style grids with sheet tabs and Word
documents as text, zoomable, built by tools/build_previews.py. The PNG
renders and screenshots are removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/samples/CTC_Partner_Map_SAMPLE.xlsx
+++ b/downloads/samples/CTC_Partner_Map_SAMPLE.xlsx
@@ -541,7 +541,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>TIER 1  (9)   Approach in the first 30 days. Can host or co-host now.</t>
+          <t>TIER 1  (9)   First wave. Can host or co-host now.</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>TIER 2  (4)   Approach at 60 to 90 days. Wants a warm intro or a track record first.</t>
+          <t>TIER 2  (4)   Second wave. Wants a warm intro or a track record first.</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>TIER 3  (2)   Later. Real, but not a first-quarter target.</t>
+          <t>TIER 3  (2)   Later. Real, but slow, large, or out of reach for now.</t>
         </is>
       </c>
     </row>

</xml_diff>